<commit_message>
Update hh-postplanner-2026-04-07.xlsx (regenerated during April 8 pipeline)
https://claude.ai/code/session_01JToKqSxpvCyeKkqfXFM9yk
</commit_message>
<xml_diff>
--- a/NBA/postplanner-imports/hh-postplanner-2026-04-07.xlsx
+++ b/NBA/postplanner-imports/hh-postplanner-2026-04-07.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>04/07/2026  11:46</t>
+          <t>04/07/2026  09:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -493,7 +493,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>04/07/2026  12:47</t>
+          <t>04/07/2026  09:30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -508,7 +508,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>04/07/2026  13:48</t>
+          <t>04/07/2026  11:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -523,7 +523,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04/07/2026  14:49</t>
+          <t>04/07/2026  11:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -537,7 +537,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04/07/2026  15:50</t>
+          <t>04/07/2026  13:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -552,7 +552,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04/07/2026  16:51</t>
+          <t>04/07/2026  13:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -567,7 +567,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04/07/2026  17:52</t>
+          <t>04/07/2026  15:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -582,7 +582,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04/07/2026  18:53</t>
+          <t>04/07/2026  16:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -597,7 +597,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04/07/2026  19:54</t>
+          <t>04/07/2026  17:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -612,7 +612,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04/07/2026  20:55</t>
+          <t>04/07/2026  19:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">

</xml_diff>